<commit_message>
Add ODM radiation calibration function
</commit_message>
<xml_diff>
--- a/docker/rsdm/template.xlsx
+++ b/docker/rsdm/template.xlsx
@@ -27,21 +27,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>样方名称</t>
   </si>
   <si>
-    <t>坐标点1</t>
-  </si>
-  <si>
-    <t>坐标点2</t>
-  </si>
-  <si>
-    <t>坐标点3</t>
-  </si>
-  <si>
-    <t>坐标点4</t>
+    <t>坐标点</t>
   </si>
   <si>
     <t>坐标中心点</t>
@@ -1191,7 +1182,8 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="12.4166666666667" customWidth="1"/>
-    <col min="2" max="34" width="18.7777777777778" customWidth="1"/>
+    <col min="2" max="2" width="39.8888888888889" customWidth="1"/>
+    <col min="3" max="31" width="18.7777777777778" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="22.5" customHeight="1" spans="1:34">
@@ -1204,99 +1196,93 @@
       <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="5" t="s">
         <v>9</v>
       </c>
       <c r="K1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="L1" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="M1" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="N1" s="6" t="s">
         <v>13</v>
       </c>
       <c r="O1" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="P1" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="Q1" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="6" t="s">
+      <c r="R1" s="7" t="s">
         <v>17</v>
       </c>
       <c r="S1" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="7" t="s">
+      <c r="T1" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="7" t="s">
+      <c r="U1" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="7" t="s">
+      <c r="V1" s="8" t="s">
         <v>21</v>
       </c>
       <c r="W1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="8" t="s">
+      <c r="X1" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="8" t="s">
+      <c r="Y1" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="8" t="s">
+      <c r="Z1" s="6" t="s">
         <v>25</v>
       </c>
       <c r="AA1" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="6" t="s">
+      <c r="AB1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="6" t="s">
+      <c r="AC1" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="6" t="s">
+      <c r="AD1" s="9" t="s">
         <v>29</v>
       </c>
       <c r="AE1" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="AG1" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="AH1" s="9" t="s">
-        <v>33</v>
-      </c>
+      <c r="AF1"/>
+      <c r="AG1"/>
+      <c r="AH1"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>